<commit_message>
agregar sistema de automatización
</commit_message>
<xml_diff>
--- a/resultados/consolidado_limpio.xlsx
+++ b/resultados/consolidado_limpio.xlsx
@@ -456,12 +456,12 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>05/06/2026</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Chaqueta impermeable</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -470,14 +470,14 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E2" t="n">
-        <v>55400</v>
+        <v>90600</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -489,45 +489,45 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>05/07/2026</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Parlante portatil</t>
+          <t>Camiseta basica</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D3" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E3" t="n">
-        <v>20200</v>
+        <v>98500</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>16/06/2026</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Camiseta basica</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
@@ -536,31 +536,31 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E4" t="n">
-        <v>107600</v>
+        <v>47800</v>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>12/07/2026</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Medias deportivas</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
@@ -569,80 +569,80 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E5" t="n">
-        <v>148600</v>
+        <v>125200</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Teclado mecanico</t>
+          <t>Camiseta basica</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D6" t="n">
         <v>5</v>
       </c>
       <c r="E6" t="n">
-        <v>40700</v>
+        <v>34000</v>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Desconocido</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>19/06/2026</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D7" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>74200</v>
+        <v>133400</v>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -654,12 +654,12 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>02/07/2026</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Audifonos Bluetooth</t>
+          <t>Parlante portatil</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -668,14 +668,14 @@
         </is>
       </c>
       <c r="D8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E8" t="n">
-        <v>175600</v>
+        <v>164400</v>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
@@ -687,12 +687,12 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>18/06/2026</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Parlante portatil</t>
+          <t>Teclado mecanico</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -701,43 +701,43 @@
         </is>
       </c>
       <c r="D9" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E9" t="n">
-        <v>110300</v>
+        <v>58100</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>29/06/2026</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Mouse inalambrico</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D10" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E10" t="n">
-        <v>156100</v>
+        <v>107500</v>
       </c>
       <c r="F10" t="inlineStr">
         <is>
@@ -746,19 +746,19 @@
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>05/07/2026</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Mouse inalambrico</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -767,14 +767,14 @@
         </is>
       </c>
       <c r="D11" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>41800</v>
+        <v>152700</v>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Desconocido</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
@@ -786,12 +786,12 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>09/06/2026</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Teclado mecanico</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
@@ -800,64 +800,64 @@
         </is>
       </c>
       <c r="D12" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E12" t="n">
-        <v>115500</v>
+        <v>65900</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>14/07/2026</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Mouse inalambrico</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D13" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E13" t="n">
-        <v>59500</v>
+        <v>80300</v>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Laura Diaz</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Desconocido</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Chaqueta impermeable</t>
+          <t>Medias deportivas</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -869,11 +869,11 @@
         <v>4</v>
       </c>
       <c r="E14" t="n">
-        <v>150600</v>
+        <v>157700</v>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
@@ -885,12 +885,12 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>12/06/2026</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Audifonos Bluetooth</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
@@ -899,92 +899,92 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E15" t="n">
-        <v>165700</v>
+        <v>144100</v>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>11/06/2026</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D16" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E16" t="n">
-        <v>80300</v>
+        <v>78100</v>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Desconocido</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>13/06/2026</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D17" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E17" t="n">
-        <v>137900</v>
+        <v>72700</v>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -1001,61 +1001,61 @@
         <v>7</v>
       </c>
       <c r="E18" t="n">
-        <v>74700</v>
+        <v>78000</v>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-01</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Parlante portatil</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D19" t="n">
         <v>2</v>
       </c>
       <c r="E19" t="n">
-        <v>40200</v>
+        <v>127500</v>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-08</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Medias deportivas</t>
+          <t>Chaqueta impermeable</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -1064,10 +1064,10 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E20" t="n">
-        <v>78000</v>
+        <v>86700</v>
       </c>
       <c r="F20" t="inlineStr">
         <is>
@@ -1076,19 +1076,19 @@
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>2026-06-01</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Parlante portatil</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -1097,14 +1097,14 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E21" t="n">
-        <v>127500</v>
+        <v>98800</v>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
@@ -1116,28 +1116,28 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>2026-06-08</t>
+          <t>2026-07-09</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Chaqueta impermeable</t>
+          <t>Parlante portatil</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="E22" t="n">
-        <v>86700</v>
+        <v>40200</v>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
@@ -1149,28 +1149,28 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Medias deportivas</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E23" t="n">
-        <v>98800</v>
+        <v>18200</v>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Laura Diaz</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
@@ -1182,28 +1182,28 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Parlante portatil</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D24" t="n">
         <v>4</v>
       </c>
       <c r="E24" t="n">
-        <v>40200</v>
+        <v>159900</v>
       </c>
       <c r="F24" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G24" t="inlineStr">
@@ -1215,12 +1215,12 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Medias deportivas</t>
+          <t>Gorra deportiva</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -1229,113 +1229,113 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E25" t="n">
-        <v>18200</v>
+        <v>36200</v>
       </c>
       <c r="F25" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E26" t="n">
-        <v>159900</v>
+        <v>174100</v>
       </c>
       <c r="F26" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Gorra deportiva</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="E27" t="n">
-        <v>36200</v>
+        <v>87300</v>
       </c>
       <c r="F27" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Desconocido</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Camiseta basica</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E28" t="n">
-        <v>174100</v>
+        <v>25600</v>
       </c>
       <c r="F28" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G28" t="inlineStr">
@@ -1347,40 +1347,40 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-15</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Medias deportivas</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E29" t="n">
-        <v>87300</v>
+        <v>26700</v>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-03</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -1394,31 +1394,31 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E30" t="n">
-        <v>25600</v>
+        <v>26700</v>
       </c>
       <c r="F30" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-14</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Medias deportivas</t>
+          <t>Gorra deportiva</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -1427,31 +1427,31 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E31" t="n">
-        <v>26700</v>
+        <v>134400</v>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Desconocido</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>2026-06-03</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -1460,31 +1460,31 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E32" t="n">
-        <v>26700</v>
+        <v>46400</v>
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Desconocido</t>
         </is>
       </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-14</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Gorra deportiva</t>
+          <t>Chaqueta impermeable</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1493,43 +1493,43 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
       <c r="E33" t="n">
-        <v>134400</v>
+        <v>92100</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Audifonos Bluetooth</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E34" t="n">
-        <v>46400</v>
+        <v>147100</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
@@ -1538,19 +1538,19 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Chaqueta impermeable</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -1559,76 +1559,76 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="E35" t="n">
-        <v>92100</v>
+        <v>38100</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Audifonos Bluetooth</t>
+          <t>Gorra deportiva</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E36" t="n">
-        <v>147100</v>
+        <v>88100</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Audifonos Bluetooth</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E37" t="n">
-        <v>38100</v>
+        <v>174900</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
@@ -1637,35 +1637,35 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Gorra deportiva</t>
+          <t>Teclado mecanico</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
       <c r="E38" t="n">
-        <v>88100</v>
+        <v>50300</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
@@ -1677,12 +1677,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Audifonos Bluetooth</t>
+          <t>Mouse inalambrico</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -1694,28 +1694,28 @@
         <v>1</v>
       </c>
       <c r="E39" t="n">
-        <v>174900</v>
+        <v>177600</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Laura Diaz</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Desconocido</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Teclado mecanico</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -1727,28 +1727,28 @@
         <v>8</v>
       </c>
       <c r="E40" t="n">
-        <v>50300</v>
+        <v>40500</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
+          <t>Laura Diaz</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Mouse inalambrico</t>
+          <t>Audifonos Bluetooth</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -1760,61 +1760,61 @@
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>177600</v>
+        <v>138400</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Medias deportivas</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E42" t="n">
-        <v>40500</v>
+        <v>24400</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Audifonos Bluetooth</t>
+          <t>Mouse inalambrico</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -1823,31 +1823,31 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E43" t="n">
-        <v>138400</v>
+        <v>126400</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Desconocido</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Medias deportivas</t>
+          <t>Camiseta basica</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -1856,14 +1856,14 @@
         </is>
       </c>
       <c r="D44" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E44" t="n">
-        <v>24400</v>
+        <v>110500</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
@@ -1875,12 +1875,12 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Mouse inalambrico</t>
+          <t>Teclado mecanico</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1889,10 +1889,10 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="E45" t="n">
-        <v>126400</v>
+        <v>169200</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
@@ -1901,19 +1901,19 @@
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1922,43 +1922,43 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>4</v>
+        <v>7</v>
       </c>
       <c r="E46" t="n">
-        <v>110500</v>
+        <v>36600</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Laura Diaz</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Desconocido</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Teclado mecanico</t>
+          <t>Camiseta basica</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E47" t="n">
-        <v>169200</v>
+        <v>55400</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -1967,52 +1967,52 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Parlante portatil</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D48" t="n">
         <v>7</v>
       </c>
       <c r="E48" t="n">
-        <v>36600</v>
+        <v>20200</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>05/06/2026</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Chaqueta impermeable</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
@@ -2024,7 +2024,7 @@
         <v>1</v>
       </c>
       <c r="E49" t="n">
-        <v>90600</v>
+        <v>107600</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
@@ -2033,19 +2033,19 @@
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Desconocido</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>05/07/2026</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -2054,64 +2054,64 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E50" t="n">
-        <v>98500</v>
+        <v>148600</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>16/06/2026</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Teclado mecanico</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="E51" t="n">
-        <v>47800</v>
+        <v>40700</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
+          <t>Laura Diaz</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>12/07/2026</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Medias deportivas</t>
+          <t>Camiseta basica</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2120,14 +2120,14 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E52" t="n">
-        <v>125200</v>
+        <v>74200</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Laura Diaz</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
@@ -2139,45 +2139,45 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>09/06/2026</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Audifonos Bluetooth</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E53" t="n">
-        <v>34000</v>
+        <v>175600</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>19/06/2026</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Parlante portatil</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -2186,43 +2186,43 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E54" t="n">
-        <v>133400</v>
+        <v>110300</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>02/07/2026</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Parlante portatil</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E55" t="n">
-        <v>164400</v>
+        <v>156100</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
@@ -2231,19 +2231,19 @@
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Desconocido</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>18/06/2026</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Teclado mecanico</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2252,31 +2252,31 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E56" t="n">
-        <v>58100</v>
+        <v>41800</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Laura Diaz</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>29/06/2026</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Mouse inalambrico</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -2285,26 +2285,26 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E57" t="n">
-        <v>107500</v>
+        <v>115500</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>05/07/2026</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -2318,14 +2318,14 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E58" t="n">
-        <v>152700</v>
+        <v>59500</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2337,78 +2337,78 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>09/06/2026</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Teclado mecanico</t>
+          <t>Chaqueta impermeable</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="E59" t="n">
-        <v>65900</v>
+        <v>150600</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Laura Diaz</t>
         </is>
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Desconocido</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>14/07/2026</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D60" t="n">
         <v>4</v>
       </c>
       <c r="E60" t="n">
-        <v>80300</v>
+        <v>165700</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>10/06/2026</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Medias deportivas</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -2417,31 +2417,31 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E61" t="n">
-        <v>157700</v>
+        <v>80300</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>12/06/2026</t>
+          <t>2026-06-09</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Audifonos Bluetooth</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2450,47 +2450,47 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E62" t="n">
-        <v>144100</v>
+        <v>137900</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>11/06/2026</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Medias deportivas</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>2</v>
+        <v>7</v>
       </c>
       <c r="E63" t="n">
-        <v>78100</v>
+        <v>74700</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2502,12 +2502,12 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>13/06/2026</t>
+          <t>2026-06-04</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Camiseta basica</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2516,10 +2516,10 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E64" t="n">
-        <v>72700</v>
+        <v>40200</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
@@ -2528,7 +2528,7 @@
       </c>
       <c r="G64" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Desconocido</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
agregar resumen ejecutivo y metricas de negocio a la automatizacion
</commit_message>
<xml_diff>
--- a/resultados/consolidado_limpio.xlsx
+++ b/resultados/consolidado_limpio.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G64"/>
+  <dimension ref="A1:G76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1479,28 +1479,28 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Chaqueta impermeable</t>
+          <t>Monitor</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E33" t="n">
-        <v>92100</v>
+        <v>750000</v>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Carlos</t>
         </is>
       </c>
       <c r="G33" t="inlineStr">
@@ -1512,28 +1512,28 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Audifonos Bluetooth</t>
+          <t>Jean</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="E34" t="n">
-        <v>147100</v>
+        <v>98000</v>
       </c>
       <c r="F34" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Maria</t>
         </is>
       </c>
       <c r="G34" t="inlineStr">
@@ -1545,45 +1545,45 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>2026-06-13</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="E35" t="n">
-        <v>38100</v>
+        <v>65000</v>
       </c>
       <c r="F35" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Carlos</t>
         </is>
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Gorra deportiva</t>
+          <t>Zapatos</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -1592,64 +1592,64 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E36" t="n">
-        <v>88100</v>
+        <v>210000</v>
       </c>
       <c r="F36" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Maria</t>
         </is>
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Audifonos Bluetooth</t>
+          <t>Chaqueta impermeable</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E37" t="n">
-        <v>174900</v>
+        <v>92100</v>
       </c>
       <c r="F37" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Teclado mecanico</t>
+          <t>Audifonos Bluetooth</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -1658,92 +1658,92 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E38" t="n">
-        <v>50300</v>
+        <v>147100</v>
       </c>
       <c r="F38" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-13</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Mouse inalambrico</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="E39" t="n">
-        <v>177600</v>
+        <v>38100</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Gorra deportiva</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E40" t="n">
-        <v>40500</v>
+        <v>88100</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -1760,44 +1760,44 @@
         <v>1</v>
       </c>
       <c r="E41" t="n">
-        <v>138400</v>
+        <v>174900</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G41" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Medias deportivas</t>
+          <t>Teclado mecanico</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="E42" t="n">
-        <v>24400</v>
+        <v>50300</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Felipe Torres</t>
         </is>
       </c>
       <c r="G42" t="inlineStr">
@@ -1809,7 +1809,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -1823,14 +1823,14 @@
         </is>
       </c>
       <c r="D43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E43" t="n">
-        <v>126400</v>
+        <v>177600</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Laura Diaz</t>
         </is>
       </c>
       <c r="G43" t="inlineStr">
@@ -1842,45 +1842,45 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Cargador USB-C</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="E44" t="n">
-        <v>110500</v>
+        <v>40500</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Laura Diaz</t>
         </is>
       </c>
       <c r="G44" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Teclado mecanico</t>
+          <t>Audifonos Bluetooth</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -1889,31 +1889,31 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E45" t="n">
-        <v>169200</v>
+        <v>138400</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G45" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Medias deportivas</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -1922,43 +1922,43 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E46" t="n">
-        <v>36600</v>
+        <v>24400</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G46" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-05</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Mouse inalambrico</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E47" t="n">
-        <v>55400</v>
+        <v>126400</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
@@ -1967,31 +1967,31 @@
       </c>
       <c r="G47" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Desconocido</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>2026-06-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Parlante portatil</t>
+          <t>Camiseta basica</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E48" t="n">
-        <v>20200</v>
+        <v>110500</v>
       </c>
       <c r="F48" t="inlineStr">
         <is>
@@ -2000,47 +2000,47 @@
       </c>
       <c r="G48" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-13</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Teclado mecanico</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E49" t="n">
-        <v>107600</v>
+        <v>169200</v>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G49" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Transferencia</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -2054,31 +2054,31 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="E50" t="n">
-        <v>148600</v>
+        <v>36600</v>
       </c>
       <c r="F50" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Laura Diaz</t>
         </is>
       </c>
       <c r="G50" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Desconocido</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Teclado mecanico</t>
+          <t>Teclado</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
@@ -2087,14 +2087,14 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="E51" t="n">
-        <v>40700</v>
+        <v>65000</v>
       </c>
       <c r="F51" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Sofia</t>
         </is>
       </c>
       <c r="G51" t="inlineStr">
@@ -2106,12 +2106,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Camiseta basica</t>
+          <t>Falda</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -2120,31 +2120,31 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E52" t="n">
-        <v>74200</v>
+        <v>52000</v>
       </c>
       <c r="F52" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Juan</t>
         </is>
       </c>
       <c r="G52" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Audifonos Bluetooth</t>
+          <t>Audifonos</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
@@ -2153,14 +2153,14 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E53" t="n">
-        <v>175600</v>
+        <v>38000</v>
       </c>
       <c r="F53" t="inlineStr">
         <is>
-          <t>Felipe Torres</t>
+          <t>Sofia</t>
         </is>
       </c>
       <c r="G53" t="inlineStr">
@@ -2172,45 +2172,45 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Parlante portatil</t>
+          <t>Chaqueta</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E54" t="n">
-        <v>110300</v>
+        <v>120000</v>
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Juan</t>
         </is>
       </c>
       <c r="G54" t="inlineStr">
         <is>
-          <t>Efectivo</t>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-02</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Camiseta basica</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -2219,31 +2219,31 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E55" t="n">
-        <v>156100</v>
+        <v>55400</v>
       </c>
       <c r="F55" t="inlineStr">
         <is>
-          <t>Camila Ruiz</t>
+          <t>Andres Gomez</t>
         </is>
       </c>
       <c r="G55" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-06</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Parlante portatil</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -2252,14 +2252,14 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E56" t="n">
-        <v>41800</v>
+        <v>20200</v>
       </c>
       <c r="F56" t="inlineStr">
         <is>
-          <t>Laura Diaz</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G56" t="inlineStr">
@@ -2271,61 +2271,61 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E57" t="n">
-        <v>115500</v>
+        <v>107600</v>
       </c>
       <c r="F57" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Sofia Mena</t>
         </is>
       </c>
       <c r="G57" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Desconocido</t>
         </is>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Mouse inalambrico</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="E58" t="n">
-        <v>59500</v>
+        <v>148600</v>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G58" t="inlineStr">
@@ -2337,24 +2337,24 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>2026-06-04</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Chaqueta impermeable</t>
+          <t>Teclado mecanico</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E59" t="n">
-        <v>150600</v>
+        <v>40700</v>
       </c>
       <c r="F59" t="inlineStr">
         <is>
@@ -2363,35 +2363,35 @@
       </c>
       <c r="G59" t="inlineStr">
         <is>
-          <t>Desconocido</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>2026-06-05</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Camiseta basica</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Electronica</t>
+          <t>Ropa</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E60" t="n">
-        <v>165700</v>
+        <v>74200</v>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Laura Diaz</t>
         </is>
       </c>
       <c r="G60" t="inlineStr">
@@ -2403,24 +2403,24 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Jean clasico</t>
+          <t>Audifonos Bluetooth</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Ropa</t>
+          <t>Electronica</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="E61" t="n">
-        <v>80300</v>
+        <v>175600</v>
       </c>
       <c r="F61" t="inlineStr">
         <is>
@@ -2429,19 +2429,19 @@
       </c>
       <c r="G61" t="inlineStr">
         <is>
-          <t>Tarjeta</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>2026-06-09</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Cargador USB-C</t>
+          <t>Parlante portatil</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -2450,31 +2450,31 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E62" t="n">
-        <v>137900</v>
+        <v>110300</v>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>Sofia Mena</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G62" t="inlineStr">
         <is>
-          <t>Transferencia</t>
+          <t>Efectivo</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-19</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Medias deportivas</t>
+          <t>Jean clasico</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -2483,14 +2483,14 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
       <c r="E63" t="n">
-        <v>74700</v>
+        <v>156100</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Andres Gomez</t>
+          <t>Camila Ruiz</t>
         </is>
       </c>
       <c r="G63" t="inlineStr">
@@ -2502,33 +2502,429 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>Cargador USB-C</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D64" t="n">
+        <v>6</v>
+      </c>
+      <c r="E64" t="n">
+        <v>41800</v>
+      </c>
+      <c r="F64" t="inlineStr">
+        <is>
+          <t>Laura Diaz</t>
+        </is>
+      </c>
+      <c r="G64" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>2026-07-15</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>Cargador USB-C</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D65" t="n">
+        <v>2</v>
+      </c>
+      <c r="E65" t="n">
+        <v>115500</v>
+      </c>
+      <c r="F65" t="inlineStr">
+        <is>
+          <t>Andres Gomez</t>
+        </is>
+      </c>
+      <c r="G65" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>2026-06-30</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>Mouse inalambrico</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>7</v>
+      </c>
+      <c r="E66" t="n">
+        <v>59500</v>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>Sofia Mena</t>
+        </is>
+      </c>
+      <c r="G66" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
           <t>2026-06-04</t>
         </is>
       </c>
-      <c r="B64" t="inlineStr">
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>Chaqueta impermeable</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>4</v>
+      </c>
+      <c r="E67" t="n">
+        <v>150600</v>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>Laura Diaz</t>
+        </is>
+      </c>
+      <c r="G67" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>2026-06-05</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Cargador USB-C</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>4</v>
+      </c>
+      <c r="E68" t="n">
+        <v>165700</v>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>Sofia Mena</t>
+        </is>
+      </c>
+      <c r="G68" t="inlineStr">
+        <is>
+          <t>Transferencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>2026-07-12</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>Jean clasico</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>8</v>
+      </c>
+      <c r="E69" t="n">
+        <v>80300</v>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>Felipe Torres</t>
+        </is>
+      </c>
+      <c r="G69" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>2026-06-09</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Cargador USB-C</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>4</v>
+      </c>
+      <c r="E70" t="n">
+        <v>137900</v>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>Sofia Mena</t>
+        </is>
+      </c>
+      <c r="G70" t="inlineStr">
+        <is>
+          <t>Transferencia</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>2026-06-28</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Medias deportivas</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>7</v>
+      </c>
+      <c r="E71" t="n">
+        <v>74700</v>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>Andres Gomez</t>
+        </is>
+      </c>
+      <c r="G71" t="inlineStr">
+        <is>
+          <t>Desconocido</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>2026-06-04</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
         <is>
           <t>Camiseta basica</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>Ropa</t>
-        </is>
-      </c>
-      <c r="D64" t="n">
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
         <v>2</v>
       </c>
-      <c r="E64" t="n">
+      <c r="E72" t="n">
         <v>40200</v>
       </c>
-      <c r="F64" t="inlineStr">
+      <c r="F72" t="inlineStr">
         <is>
           <t>Andres Gomez</t>
         </is>
       </c>
-      <c r="G64" t="inlineStr">
+      <c r="G72" t="inlineStr">
         <is>
           <t>Desconocido</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>Laptop</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D73" t="n">
+        <v>1</v>
+      </c>
+      <c r="E73" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="F73" t="inlineStr">
+        <is>
+          <t>Carlos</t>
+        </is>
+      </c>
+      <c r="G73" t="inlineStr">
+        <is>
+          <t>Efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>2026-08-25</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Camisa</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D74" t="n">
+        <v>3</v>
+      </c>
+      <c r="E74" t="n">
+        <v>45000</v>
+      </c>
+      <c r="F74" t="inlineStr">
+        <is>
+          <t>Ana</t>
+        </is>
+      </c>
+      <c r="G74" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Mouse</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>Electronica</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>4</v>
+      </c>
+      <c r="E75" t="n">
+        <v>35000</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Diego</t>
+        </is>
+      </c>
+      <c r="G75" t="inlineStr">
+        <is>
+          <t>Efectivo</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>2026-08-27</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Pantalon</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>Ropa</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>2</v>
+      </c>
+      <c r="E76" t="n">
+        <v>89000</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Ana</t>
+        </is>
+      </c>
+      <c r="G76" t="inlineStr">
+        <is>
+          <t>Tarjeta</t>
         </is>
       </c>
     </row>

</xml_diff>